<commit_message>
cross neo selective ensemble policy lock
- make fast ESM2 QK gate metrics reproducible from persisted scores

- add v2.1 selective routing policy with abstention tables

- add unique pMHC wetlab prioritization table for TCR branch

Co-Authored-By: Codex <codex@openai.com>
</commit_message>
<xml_diff>
--- a/project/results/cross_neo_v2_sota_sprint_2026_05_09/CROSS_Neo_v2_all_results_summary_plus_runpod_esm2_fast_gate.xlsx
+++ b/project/results/cross_neo_v2_sota_sprint_2026_05_09/CROSS_Neo_v2_all_results_summary_plus_runpod_esm2_fast_gate.xlsx
@@ -27396,16 +27396,16 @@
         <v>0.2359550561797753</v>
       </c>
       <c r="F422">
-        <v>0.6453994509447532</v>
+        <v>0.636884934026875</v>
       </c>
       <c r="G422">
-        <v>0.7601540616246498</v>
+        <v>0.759453781512605</v>
       </c>
       <c r="H422">
-        <v>0.2261710541951407</v>
+        <v>0.2261710541951304</v>
       </c>
       <c r="I422">
-        <v>0.2765216454783633</v>
+        <v>0.276521645478337</v>
       </c>
       <c r="J422">
         <v>1</v>
@@ -27464,10 +27464,10 @@
         <v>0.7223389355742296</v>
       </c>
       <c r="H423">
-        <v>0.2667074225583094</v>
+        <v>0.2667074225583097</v>
       </c>
       <c r="I423">
-        <v>0.3038769112357117</v>
+        <v>0.3038769112357079</v>
       </c>
       <c r="J423">
         <v>0.8</v>
@@ -27526,10 +27526,10 @@
         <v>0.7865497076023391</v>
       </c>
       <c r="H424">
-        <v>0.251533702682972</v>
+        <v>0.251533702683007</v>
       </c>
       <c r="I424">
-        <v>0.3121032576995686</v>
+        <v>0.3121032576995555</v>
       </c>
       <c r="J424">
         <v>0.6</v>
@@ -27588,10 +27588,10 @@
         <v>0.6645658263305322</v>
       </c>
       <c r="H425">
-        <v>0.2665246757819558</v>
+        <v>0.2665246757819807</v>
       </c>
       <c r="I425">
-        <v>0.2755317328440054</v>
+        <v>0.2755317328440225</v>
       </c>
       <c r="J425">
         <v>0.8</v>
@@ -27680,7 +27680,7 @@
         <v>0.7</v>
       </c>
       <c r="E2">
-        <v>0.6453994509447532</v>
+        <v>0.636884934026875</v>
       </c>
       <c r="F2">
         <v>0.7</v>
@@ -27689,7 +27689,7 @@
         <v>77</v>
       </c>
       <c r="H2">
-        <v>0.6453994509447532</v>
+        <v>0.636884934026875</v>
       </c>
       <c r="I2">
         <v>0.7</v>
@@ -27877,16 +27877,16 @@
         <v>0.2359550561797753</v>
       </c>
       <c r="H2">
-        <v>0.6453994509447532</v>
+        <v>0.636884934026875</v>
       </c>
       <c r="I2">
-        <v>0.7601540616246498</v>
+        <v>0.759453781512605</v>
       </c>
       <c r="J2">
-        <v>0.2261710541951407</v>
+        <v>0.2261710541951304</v>
       </c>
       <c r="K2">
-        <v>0.2765216454783633</v>
+        <v>0.276521645478337</v>
       </c>
       <c r="L2">
         <v>1</v>
@@ -27945,10 +27945,10 @@
         <v>0.7223389355742296</v>
       </c>
       <c r="J3">
-        <v>0.2667074225583094</v>
+        <v>0.2667074225583097</v>
       </c>
       <c r="K3">
-        <v>0.3038769112357117</v>
+        <v>0.3038769112357079</v>
       </c>
       <c r="L3">
         <v>0.8</v>
@@ -28007,10 +28007,10 @@
         <v>0.7865497076023391</v>
       </c>
       <c r="J4">
-        <v>0.251533702682972</v>
+        <v>0.251533702683007</v>
       </c>
       <c r="K4">
-        <v>0.3121032576995686</v>
+        <v>0.3121032576995555</v>
       </c>
       <c r="L4">
         <v>0.6</v>
@@ -28069,10 +28069,10 @@
         <v>0.6645658263305322</v>
       </c>
       <c r="J5">
-        <v>0.2665246757819558</v>
+        <v>0.2665246757819807</v>
       </c>
       <c r="K5">
-        <v>0.2755317328440054</v>
+        <v>0.2755317328440225</v>
       </c>
       <c r="L5">
         <v>0.8</v>

</xml_diff>